<commit_message>
Re-did parts of bom
</commit_message>
<xml_diff>
--- a/MotorDriver1/jlcpcb/production_files_final/BOM-MotorDriver1.xlsx
+++ b/MotorDriver1/jlcpcb/production_files_final/BOM-MotorDriver1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emma/Documents/JHU/Capstone_Smart_Saddle_Pad/MotorDriver1/jlcpcb/production_files_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715045A6-7FB7-9049-83F9-FD002F038A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C0A2EA-03A1-A745-A896-4F20B260302E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{24B93369-4AC7-7947-B738-BCC767C42009}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" xr2:uid="{24B93369-4AC7-7947-B738-BCC767C42009}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM-MotorDriver1" sheetId="1" r:id="rId1"/>
@@ -79,9 +79,6 @@
     <t>C_0402_1005Metric</t>
   </si>
   <si>
-    <t>C1524</t>
-  </si>
-  <si>
     <t>100 nF</t>
   </si>
   <si>
@@ -112,9 +109,6 @@
     <t>C8</t>
   </si>
   <si>
-    <t>C1705</t>
-  </si>
-  <si>
     <t>47 nF</t>
   </si>
   <si>
@@ -266,13 +260,19 @@
   </si>
   <si>
     <t>C77012</t>
+  </si>
+  <si>
+    <t>C19666</t>
+  </si>
+  <si>
+    <t>C15195</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -405,12 +405,6 @@
       <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -755,9 +749,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1218,7 +1211,7 @@
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -1226,16 +1219,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s">
         <v>20</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6">
         <v>9</v>
@@ -1243,16 +1236,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7">
         <v>10</v>
@@ -1263,13 +1256,13 @@
         <v>120</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -1277,16 +1270,16 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
       </c>
       <c r="C9" t="s">
         <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -1294,16 +1287,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>81</v>
+      <c r="D10" t="s">
+        <v>79</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -1311,16 +1304,16 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -1328,16 +1321,16 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
         <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -1345,16 +1338,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
         <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -1362,16 +1355,16 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" t="s">
         <v>42</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>43</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
-        <v>45</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -1379,16 +1372,16 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" t="s">
         <v>46</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" t="s">
-        <v>49</v>
       </c>
       <c r="E15">
         <v>3</v>
@@ -1396,16 +1389,16 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" t="s">
         <v>50</v>
       </c>
-      <c r="B16" t="s">
+      <c r="D16" t="s">
         <v>51</v>
-      </c>
-      <c r="C16" t="s">
-        <v>52</v>
-      </c>
-      <c r="D16" t="s">
-        <v>53</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -1413,16 +1406,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" t="s">
         <v>54</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
         <v>55</v>
-      </c>
-      <c r="C17" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" t="s">
-        <v>57</v>
       </c>
       <c r="E17">
         <v>4</v>
@@ -1430,16 +1423,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" t="s">
         <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" t="s">
-        <v>60</v>
       </c>
       <c r="E18">
         <v>3</v>
@@ -1447,16 +1440,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
         <v>61</v>
       </c>
-      <c r="B19" t="s">
+      <c r="D19" t="s">
         <v>62</v>
-      </c>
-      <c r="C19" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" t="s">
-        <v>64</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1464,16 +1457,16 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
         <v>66</v>
-      </c>
-      <c r="C20" t="s">
-        <v>67</v>
-      </c>
-      <c r="D20" t="s">
-        <v>68</v>
       </c>
       <c r="E20">
         <v>2</v>
@@ -1481,16 +1474,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
         <v>69</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
         <v>70</v>
-      </c>
-      <c r="C21" t="s">
-        <v>71</v>
-      </c>
-      <c r="D21" t="s">
-        <v>72</v>
       </c>
       <c r="E21">
         <v>1</v>
@@ -1498,16 +1491,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" t="s">
         <v>73</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
         <v>74</v>
-      </c>
-      <c r="C22" t="s">
-        <v>75</v>
-      </c>
-      <c r="D22" t="s">
-        <v>76</v>
       </c>
       <c r="E22">
         <v>4</v>
@@ -1515,16 +1508,16 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>75</v>
+      </c>
+      <c r="B23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" t="s">
         <v>77</v>
       </c>
-      <c r="B23" t="s">
+      <c r="D23" t="s">
         <v>78</v>
-      </c>
-      <c r="C23" t="s">
-        <v>79</v>
-      </c>
-      <c r="D23" t="s">
-        <v>80</v>
       </c>
       <c r="E23">
         <v>1</v>

</xml_diff>